<commit_message>
Update ACMG Excel template with revised 15 variants review
</commit_message>
<xml_diff>
--- a/ACMG_EVIDENCE_REVIEW/ACMG_AMP_15_Variants_Template11,, (2).xlsx
+++ b/ACMG_EVIDENCE_REVIEW/ACMG_AMP_15_Variants_Template11,, (2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kholu\Downloads\38833FF26BA1D.UnigramPreview_g9c9v27vpyspw!App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CE6984F-E6EB-4415-AD93-87DBD10BAB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3E40E4D-EC88-4471-BC05-2C478FF4B6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="300">
   <si>
     <t>ACMG/AMP VARIANT REVIEW — 15 SELECTED VARIANTS</t>
   </si>
@@ -1190,9 +1190,6 @@
     <t>[18] National Center for Biotechnology Information. (n.d.). ClinVar: BRCA2 Variation ID 2574093. https://www.ncbi.nlm.nih.gov/clinvar/variation/2574093/</t>
   </si>
   <si>
-    <t>NM_024675.4 c.3515T&gt;G p.Leu1172Arg</t>
-  </si>
-  <si>
     <t>VEP Consequence:
 missense_variant
 Impact: MODERATE</t>
@@ -1201,96 +1198,15 @@
     <t>missense_variant</t>
   </si>
   <si>
-    <t>PM2_Supporting</t>
-  </si>
-  <si>
     <t>Supporting</t>
   </si>
   <si>
-    <t xml:space="preserve">16:603570 A&gt;G  </t>
-  </si>
-  <si>
-    <t>Likely pathogenic; criteria_provided, single_submitter.
-ClinVar lists this variant as Likely pathogenic based on a single submitter. The review status indicates “criteria provided, single submitter,” meaning the classification is not expert‑panel reviewed. The ClinVar classification is external and must not be used as ACMG/AMP evidence unless independently supported by project data.</t>
-  </si>
-  <si>
-    <t>GNOMAD_STATUS: NOT_FOUND; GNOMAD_EXOME_AF: .; GNOMAD_GENOME_AF: .
-The project annotation reports NOT_FOUND for both exome and genome datasets. Missing AF values must not be interpreted as zero. The absence of a matching record does not confirm absence from the population. PM2 cannot be applied at a strong level based on NOT_FOUND alone.</t>
-  </si>
-  <si>
-    <t>deleterious.
-SIFT predicts that the amino acid substitution may negatively affect protein function. This prediction supports potential functional impact but is considered supporting evidence only and cannot independently establish pathogenicity.</t>
-  </si>
-  <si>
-    <t>probably_damaging.
-PolyPhen‑2 predicts the variant is likely damaging. As with SIFT, this prediction is supportive but not sufficient for strong ACMG/AMP criteria without additional evidence.</t>
-  </si>
-  <si>
-    <t>The variant is extremely rare in population databases. gnomAD returned NOT_FOUND for both exome and genome datasets. Computational predictions (SIFT deleterious; PolyPhen probably damaging) support a possible functional impact. No functional, segregation, or case-level evidence was identified in the project dataset.</t>
-  </si>
-  <si>
-    <t>The missense change p.Leu1172Arg occurs in PALB2, a gene associated with hereditary cancer‑predisposing syndromes. Although computational predictions suggest a possible damaging effect, no functional studies or clinical evidence were found. The ClinVar classification is single‑submitter and cannot be used as strong evidence. Therefore, PM2_Supporting is the only applicable criterion.</t>
-  </si>
-  <si>
     <t>ClinVar (CLNSIG, CLNREVSTAT, CLNDN); VEP MANE annotation (HGVS, consequence, impact); gnomAD query status; SIFT and PolyPhen predictions; final_annotation_with_VEP_SIFT_PolyPhen.tsv.</t>
   </si>
   <si>
-    <t>No functional studies available. No segregation or case-level evidence. gnomAD NOT_FOUND cannot be interpreted as AF = 0. ClinVar classification is single‑submitter. Computational predictions alone cannot establish pathogenicity. Evidence is insufficient to support LP or P classification.</t>
-  </si>
-  <si>
-    <t>VUS — Variant of Uncertain Significance.
-Only PM2_Supporting is met. Evidence is insufficient to classify the variant as Likely Pathogenic or Pathogenic.</t>
-  </si>
-  <si>
-    <t>ClinVar reports Likely pathogenic (single submitter). The project’s independent ACMG/AMP assessment remains VUS due to limited evidence. The difference reflects the absence of functional, segregation, or strong population data in the project dataset.</t>
-  </si>
-  <si>
-    <t>16:603594 G&gt;A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NM_024675.4  c.3431T&gt;C:p.Leu1144Pro.
-</t>
-  </si>
-  <si>
-    <t>Pathogenic; criteria_provided, multiple_submitters, no_conflicts.
-ClinVar lists this variant as Pathogenic with multiple submitters and no conflicts. This classification is external and must not be used as ACMG/AMP evidence unless independently supported by project data. The review status indicates that multiple laboratories provided consistent interpretations.</t>
-  </si>
-  <si>
-    <t>GNOMAD_STATUS: FOUND; GNOMAD_EXOME_AF = 6.840497386245948e-07; GNOMAD_GENOME_AF = .
-The project annotation reports a very low exome allele frequency and a missing genome AF. Missing AF values must not be interpreted as zero. The extremely low exome AF supports rarity but does not independently establish pathogenicity. PM2_Supporting may be considered when combined with additional evidence.</t>
-  </si>
-  <si>
-    <t>PM2_Supporting.</t>
-  </si>
-  <si>
-    <t>Supporting.</t>
-  </si>
-  <si>
-    <t>The variant is extremely rare in population databases. gnomAD exome AF is 6.84e-07, and genome AF is missing. Computational predictions (SIFT deleterious; PolyPhen probably damaging) support a possible functional impact. No functional, segregation, or case-level evidence was identified in the project dataset.</t>
-  </si>
-  <si>
-    <t>The missense change p.Leu1144Pro occurs in PALB2, a gene associated with hereditary cancer‑predisposing syndromes. Although computational predictions suggest a possible damaging effect, no functional studies or clinical evidence were found. The ClinVar classification is based on multiple submitters but cannot be used as strong evidence without independent verification. Therefore, PM2_Supporting is the only applicable criterion.</t>
-  </si>
-  <si>
-    <t>No functional studies available. No segregation or case-level evidence. gnomAD genome AF missing. Computational predictions alone cannot establish pathogenicity. Evidence is insufficient to support LP or P classification independently of ClinVar.</t>
-  </si>
-  <si>
-    <t>ClinVar reports Pathogenic (multiple submitters, no conflicts). The project’s independent ACMG/AMP assessment remains VUS due to limited evidence. The difference reflects the absence of functional, segregation, or strong population data in the project dataset.</t>
-  </si>
-  <si>
-    <t>16:603505 C&gt;A</t>
-  </si>
-  <si>
-    <t>NM_024675.4 c.3431T&gt;C :p.Leu1144Pro</t>
-  </si>
-  <si>
     <t>Uncertain significance; criteria_provided, single_submitter</t>
   </si>
   <si>
-    <t>GNOMAD_STATUS: NOT_FOUND; GNOMAD_EXOME_AF: .; GNOMAD_GENOME_AF: .
-Missing AF values must not be interpreted as zero; NOT_FOUND does not prove absence from the population.</t>
-  </si>
-  <si>
     <t>missense_variant; MODERATE</t>
   </si>
   <si>
@@ -1300,22 +1216,261 @@
     <t>probably_damaging</t>
   </si>
   <si>
-    <t>The variant is extremely rare in gnomAD (NOT_FOUND for both exome and genome datasets). Computational predictions (SIFT deleterious; PolyPhen probably damaging) suggest possible impact on PALB2 protein function, but no functional, segregation, or case-level data are available.</t>
-  </si>
-  <si>
-    <t>PALB2 is a gene associated with hereditary cancer-predisposing syndromes. For this missense variant, rarity supports PM2_Supporting, and damaging computational predictions provide only supporting evidence. In the absence of functional studies, segregation data, or strong clinical evidence, no additional ACMG/AMP criteria can be confidently applied.</t>
-  </si>
-  <si>
     <t>ClinVar (PALB2 Variation ID 1372173); final_annotation_with_VEP_SIFT_PolyPhen.tsv (VEP consequence, impact, SIFT, PolyPhen, gnomAD status); ACMG/AMP guidelines (Richards et al., 2015); VEP methodology (McLaren et al., 2016); gnomAD database (Broad Institute).</t>
   </si>
   <si>
-    <t>No functional assays, segregation data, or case-level evidence are available. gnomAD NOT_FOUND cannot be treated as AF = 0. ClinVar classification is based on a single submitter and is not expert-panel evidence. Computational predictions alone are insufficient to establish pathogenicity.</t>
-  </si>
-  <si>
-    <t>VUS — Variant of Uncertain Significance</t>
-  </si>
-  <si>
-    <t>ClinVar: Uncertain significance (single submitter). Project ACMG/AMP assessment: VUS, consistent with limited available evidence.</t>
+    <t>17:7674903:TTC&gt;T</t>
+  </si>
+  <si>
+    <t>NM_000546.6:c.626_627del (p.Arg209LysfsTer6). MANE Select ENST00000269305.9. [6, 23, 24]</t>
+  </si>
+  <si>
+    <t>Pathogenic; criteria provided, multiple submitters, no conflicts</t>
+  </si>
+  <si>
+    <t>FOUND. Project gnomAD exome AF = 6.840459952527208e-7; genome AF unavailable. Rarity is documented, but PM2_Supporting is not assigned because ancestry-level counts/frequencies and quality information were not provided. Missing AF is not zero. [7, 22, 23]</t>
+  </si>
+  <si>
+    <t>frameshift_variant; HIGH</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>PVS1. [22, 25]</t>
+  </si>
+  <si>
+    <t>Very Strong (+8 points). [22]</t>
+  </si>
+  <si>
+    <t>The MANE frameshift p.Arg209LysfsTer6 introduces a premature stop at approximately residue 214, upstream of Lys351. The TP53 PVS1 flowchart predicts nonsense-mediated decay. [6, 23–25]</t>
+  </si>
+  <si>
+    <t>The early premature stop meets PVS1 at Very Strong strength. No additional criteria were established. Under the TP53 v2.4 point framework, 8 points supports Likely Pathogenic. ClinVar and prioritization scores were excluded from the evidence assessment. [5, 22, 25]</t>
+  </si>
+  <si>
+    <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; PVS1 flowchart [25]. ClinVar [19]: external comparison only.</t>
+  </si>
+  <si>
+    <t>NMD is predicted rather than experimentally confirmed. Ancestry-specific population data and independently reviewed case or segregation evidence were unavailable. PM2 was not assigned. [22–25]</t>
+  </si>
+  <si>
+    <t>Likely Pathogenic. PVS1 (Very Strong): 8 points under ClinGen TP53 v2.4. [22, 25]</t>
+  </si>
+  <si>
+    <t>ClinVar reports Pathogenic. The project assessment is Likely Pathogenic because the reviewed evidence totals 8 points, below the Pathogenic threshold of ≥10. [19, 22, 25]</t>
+  </si>
+  <si>
+    <t>17:7670656:CT&gt;C</t>
+  </si>
+  <si>
+    <t>NM_000546.6:c.1052del (p.Lys351ArgfsTer19). MANE Select ENST00000269305.9. [6, 23, 24]</t>
+  </si>
+  <si>
+    <t>Likely pathogenic; criteria provided, single submitter</t>
+  </si>
+  <si>
+    <t>NOT_FOUND (Does not mean AF=0). Exome and genome AF missing; re-query and r3 final review also report NOT_FOUND.</t>
+  </si>
+  <si>
+    <t>PVS1_Moderate. [22, 25]</t>
+  </si>
+  <si>
+    <t>Moderate (+2 points). [22, 25]</t>
+  </si>
+  <si>
+    <t>The MANE frameshift p.Lys351ArgfsTer19 introduces a new stop at approximately residue 369. This stop falls within the Gly356–Asp393 branch of the TP53 PVS1 flowchart, with predicted NMD escape. [23–25]</t>
+  </si>
+  <si>
+    <t>The position of the new stop supports PVS1_Moderate rather than PVS1 at Very Strong strength. NOT_FOUND does not justify PM2. The resulting 2 points supports VUS under TP53 v2.4. [5, 22, 25]</t>
+  </si>
+  <si>
+    <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; PVS1 flowchart [25]. ClinVar [20]: external comparison only.</t>
+  </si>
+  <si>
+    <t>Population frequencies are unavailable; NOT_FOUND does not establish absence. NMD escape is predicted. Functional, segregation and case-level evidence were not independently scored. [22–25]</t>
+  </si>
+  <si>
+    <t>VUS — Variant of Uncertain Significance. PVS1_Moderate: 2 points under ClinGen TP53 v2.4. [22, 25]</t>
+  </si>
+  <si>
+    <t>ClinVar reports Likely Pathogenic. The project assessment remains VUS because PVS1_Moderate alone provides 2 points, insufficient for Likely Pathogenic. [20, 22, 25]</t>
+  </si>
+  <si>
+    <t>17:7675107:T&gt;C</t>
+  </si>
+  <si>
+    <t>MANE Select: NM_000546.6
+ENST00000269305.9:c.505A&gt;G
+ENSP00000269305.4:p.Met169Val</t>
+  </si>
+  <si>
+    <t>Uncertain significance; criteria provided, multiple submitters, no conflicts</t>
+  </si>
+  <si>
+    <t>FOUND. Project gnomAD exome AF = 1.368095733867073e-6; genome AF unavailable. PM2_Supporting not assigned because ancestry-level counts/frequencies and quality information were not supplied. Missing AF is not zero. [7, 22, 23]</t>
+  </si>
+  <si>
+    <t>tolerated</t>
+  </si>
+  <si>
+    <t>NA (not available in project output)</t>
+  </si>
+  <si>
+    <t>BS3_Supporting; BP4_Moderate. [22, 26, 27]</t>
+  </si>
+  <si>
+    <t>BS3_Supporting: Supporting (−1 point). BP4_Moderate: Moderate (−2 points). Total = −3. [22]</t>
+  </si>
+  <si>
+    <t>ClinGen Table S3 reports M169V as partially functional in Kato and noLOF in Funk, Giacomelli and Kotler (BS3_Supporting). Table S2 reports aGVGD C0, BayesDel −0.0177298 and SpliceAI 0 (BP4_Moderate). [26, 27]</t>
+  </si>
+  <si>
+    <t>The functional results support BS3_Supporting (−1). BayesDel, aGVGD and SpliceAI meet BP4_Moderate (−2). The total of −3 supports Likely Benign under TP53 v2.4. SIFT was not counted separately; PM2 was not assigned from aggregate AF alone. [22, 26, 27]</t>
+  </si>
+  <si>
+    <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; functional Table S3 [26]; bioinformatic Table S2 [27]. ClinVar [21]: external comparison only.</t>
+  </si>
+  <si>
+    <t>ClinGen supplemental codes are preliminary and were checked against TP53 rule conditions. SpliceAI is predictive, not an RNA assay. No case-level evidence was scored. Additional evidence could change the assessment. [22, 26, 27]</t>
+  </si>
+  <si>
+    <t>Likely Benign. BS3_Supporting (−1) + BP4_Moderate (−2) = −3 points under ClinGen TP53 v2.4. [22, 26, 27]</t>
+  </si>
+  <si>
+    <t>ClinVar project snapshot reports VUS. The project assessment is Likely Benign based on reviewed ClinGen functional and computational evidence. ClinVar was used only for comparison. [21, 22, 26, 27]</t>
+  </si>
+  <si>
+    <t>[19] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 372539. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/372539/</t>
+  </si>
+  <si>
+    <t>[20] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 1066207. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/1066207/</t>
+  </si>
+  <si>
+    <t>[21] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 844926. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/844926/</t>
+  </si>
+  <si>
+    <t>[22] ClinGen TP53 Variant Curation Expert Panel. (n.d.). ClinGen TP53 Expert Panel specifications to the ACMG/AMP variant interpretation guidelines for TP53 (Version 2.4; GN009). Clinical Genome Resource. Retrieved October 24, 2026, from https://cspec.genome.network/cspec/ui/svi/svi/GN009</t>
+  </si>
+  <si>
+    <t>[23] Graduation project team. (n.d.). Variant Prioritization + Scoring Final A [Unpublished project dataset and methodology]. Supplied ZIP archive. Sources: input/final_annotation_with_VEP_SIFT_PolyPhen.tsv; results/11_merged_VEP_ClinVar_gnomAD_CORRECTED.tsv; results/14_gnomad_r3_final_review.tsv; results/prioritized_variants_CORRECTED.tsv; docs/variant_prioritization_methods.md. Scores represent educational prioritization, not independent ACMG/AMP classifications.</t>
+  </si>
+  <si>
+    <t>[24] Graduation project team. (n.d.). Graduation_Project_Final [Unpublished project annotation dataset]. Supplied ZIP archive. Sources: results/tables/clinvar_annotations.tsv; results/tables/final_annotation_with_VEP.tsv. ClinVar assertions are the project snapshots, not a live database reassessment.</t>
+  </si>
+  <si>
+    <t>[25] ClinGen TP53 Variant Curation Expert Panel. (n.d.). PVS1 flowchart for TP53 null variants in relation to NM_000546.6 [Flowchart, Version 2.4 supporting file]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/a59085f9-6c52-4c36-9c42-159f3f2c3694/data</t>
+  </si>
+  <si>
+    <t>[26] ClinGen TP53 Variant Curation Expert Panel. (n.d.). Supplementary Table S3: Functional results for selected assays and corresponding preliminary PS3 and BS3 codes for every possible p53 missense variant using the TP53 specifications v2 [Data set]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/f7b4de92-567a-497d-a8db-0f673c8bb36c/data</t>
+  </si>
+  <si>
+    <t>[27] ClinGen TP53 Variant Curation Expert Panel. (n.d.). Supplementary Table S2: Bioinformatic predictions and corresponding PP3 and BP4 codes for every possible p53 missense variant using the TP53 specifications v2 [Data set]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/f24d9c2f-5cb4-4c1a-bdf6-7d73331fc77b/data</t>
+  </si>
+  <si>
+    <t>16:23603570 AA&gt;GAG</t>
+  </si>
+  <si>
+    <t>NM_024675.4:c.3448_3450delinsTT; p.Leu1150PhefsTer13</t>
+  </si>
+  <si>
+    <t>gnomAD status: NOT_FOUND; genome and exome AF recorded as . (no frequency values reported)</t>
+  </si>
+  <si>
+    <t>Not applicable (frameshift variant)</t>
+  </si>
+  <si>
+    <t>VEP consequence: frameshift_variant;                    impact: HIGH</t>
+  </si>
+  <si>
+    <t>PVS1</t>
+  </si>
+  <si>
+    <t>Very Strong</t>
+  </si>
+  <si>
+    <t>The variant introduces a frameshift and premature termination codon (p.Leu1150PhefsTer13), consistent with PALB2 loss‑of‑function mechanism.</t>
+  </si>
+  <si>
+    <t>PALB2 is a tumor‑suppressor gene where loss‑of‑function is an established disease mechanism. Frameshift variants upstream of the final exon are predicted to undergo NMD. This deletion‑insertion disrupts coding sequence and produces a truncated protein.</t>
+  </si>
+  <si>
+    <t>gnomAD “NOT_FOUND” does not confirm absence; no functional assay available for this exact variant.</t>
+  </si>
+  <si>
+    <t>Pathogenic (PVS1 Very Strong)</t>
+  </si>
+  <si>
+    <t>ClinVar reports Likely pathogenic; project classification is Pathogenic based on PVS1 Very Strong.</t>
+  </si>
+  <si>
+    <t>16:23603589 G&gt;A</t>
+  </si>
+  <si>
+    <t>NM_024675.4:c.3431T&gt;C; p.Leu1144Pro</t>
+  </si>
+  <si>
+    <t>Uncertain significance; criteria provided, single submitter</t>
+  </si>
+  <si>
+    <t>Exome AF ≈ 5.6840497e‑05; Genome AF “.”; Status: FOUND (very low frequency)</t>
+  </si>
+  <si>
+    <t>probably damaging</t>
+  </si>
+  <si>
+    <t>PM2</t>
+  </si>
+  <si>
+    <t>Variant observed at extremely low frequency in gnomAD exomes.</t>
+  </si>
+  <si>
+    <t>Rarity supports pathogenicity under ACMG/AMP PM2‑Supporting, but does not independently establish disease association.</t>
+  </si>
+  <si>
+    <t>No functional evidence; no segregation data; rarity alone insufficient for LP/P.</t>
+  </si>
+  <si>
+    <t>VUS</t>
+  </si>
+  <si>
+    <t>ClinVar = VUS; project classification = VUS (agreement).</t>
+  </si>
+  <si>
+    <t>16:23603505 C&gt;A</t>
+  </si>
+  <si>
+    <t>NM_024675.4:c.3515T&gt;G; p.Leu1172Arg</t>
+  </si>
+  <si>
+    <t>Genome AF: “.”; Exome AF: “.”; Status: NOT_FOUND (missing ≠ zero)</t>
+  </si>
+  <si>
+    <t>PP3</t>
+  </si>
+  <si>
+    <t>Both SIFT and PolyPhen‑2 predict a damaging effect for p.Leu1172Arg.</t>
+  </si>
+  <si>
+    <t>Computational evidence suggests a deleterious impact on PALB2 protein structure; however, computational evidence alone cannot establish pathogenicity.</t>
+  </si>
+  <si>
+    <t>No functional assay available; ClinVar classifies the variant as VUS; computational predictions are supporting only.</t>
+  </si>
+  <si>
+    <t>ClinVar reports VUS; project classification agrees (VUS).</t>
+  </si>
+  <si>
+    <t>[28] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: PALB2 Variation ID 1731521.  https://www.ncbi.nlm.nih.gov/clinvar/variation/1731521/ (ncbi.nlm.nih.gov in Bing)</t>
+  </si>
+  <si>
+    <t>[29] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: PALB2 Variation ID 628361.</t>
+  </si>
+  <si>
+    <t>[30] Broad Institute. (n.d.). gnomAD: The Genome Aggregation Database.  https://gnomad.broadinstitute.org/</t>
+  </si>
+  <si>
+    <t>[31] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: PALB2 Variation ID 1372173. https://www.ncbi.nlm.nih.gov/clinvar/variation/1372173/ (ncbi.nlm.nih.gov in Bing)</t>
   </si>
 </sst>
 </file>
@@ -1534,15 +1689,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1872,48 +2027,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="19.8">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
     </row>
     <row r="4" spans="1:18" ht="27.6">
       <c r="A4" s="1" t="s">
@@ -2483,55 +2638,55 @@
         <v>31</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>212</v>
+        <v>265</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>207</v>
+        <v>266</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>209</v>
+        <v>98</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>214</v>
+        <v>267</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>208</v>
+        <v>269</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>215</v>
+        <v>268</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>216</v>
+        <v>268</v>
       </c>
       <c r="K14" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="L14" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="O14" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="L14" s="20" t="s">
-        <v>211</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="N14" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="O14" s="4" t="s">
-        <v>219</v>
-      </c>
       <c r="P14" s="4" t="s">
-        <v>220</v>
+        <v>274</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>221</v>
+        <v>275</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="165.6">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="69">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -2539,52 +2694,52 @@
         <v>32</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>223</v>
+        <v>277</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>224</v>
+        <v>278</v>
       </c>
       <c r="E15" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="L15" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>228</v>
-      </c>
       <c r="M15" s="4" t="s">
-        <v>229</v>
+        <v>283</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>230</v>
+        <v>284</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>231</v>
+        <v>285</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>232</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="130.80000000000001" customHeight="1">
@@ -2595,318 +2750,220 @@
         <v>33</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>233</v>
+        <v>288</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>234</v>
+        <v>289</v>
       </c>
       <c r="E16" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="L16" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="L16" s="4" t="s">
-        <v>211</v>
-      </c>
       <c r="M16" s="4" t="s">
-        <v>240</v>
+        <v>292</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>241</v>
+        <v>293</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>244</v>
+        <v>286</v>
       </c>
       <c r="R16" s="4" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="96.6">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17:7674903:TTC&gt;T</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NM_000546.6:c.626_627del (p.Arg209LysfsTer6). MANE Select ENST00000269305.9. [6, 23, 24]</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">frameshift_variant</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pathogenic; criteria provided, multiple submitters, no conflicts</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FOUND. Project gnomAD exome AF = 6.840459952527208e-7; genome AF unavailable. Rarity is documented, but PM2_Supporting is not assigned because ancestry-level counts/frequencies and quality information were not provided. Missing AF is not zero. [7, 22, 23]</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">frameshift_variant; HIGH</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not applicable</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not applicable</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PVS1. [22, 25]</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Very Strong (+8 points). [22]</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>The MANE frameshift p.Arg209LysfsTer6 introduces a premature stop at approximately residue 214, upstream of Lys351. The TP53 PVS1 flowchart predicts nonsense-mediated decay. [6, 23–25]</t>
-        </is>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>The early premature stop meets PVS1 at Very Strong strength. No additional criteria were established. Under the TP53 v2.4 point framework, 8 points supports Likely Pathogenic. ClinVar and prioritization scores were excluded from the evidence assessment. [5, 22, 25]</t>
-        </is>
-      </c>
-      <c r="O17" s="4" t="inlineStr">
-        <is>
-          <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; PVS1 flowchart [25]. ClinVar [19]: external comparison only.</t>
-        </is>
-      </c>
-      <c r="P17" s="4" t="inlineStr">
-        <is>
-          <t>NMD is predicted rather than experimentally confirmed. Ancestry-specific population data and independently reviewed case or segregation evidence were unavailable. PM2 was not assigned. [22–25]</t>
-        </is>
-      </c>
-      <c r="Q17" s="4" t="inlineStr">
-        <is>
-          <t>Likely Pathogenic. PVS1 (Very Strong): 8 points under ClinGen TP53 v2.4. [22, 25]</t>
-        </is>
-      </c>
-      <c r="R17" s="4" t="inlineStr">
-        <is>
-          <t>ClinVar reports Pathogenic. The project assessment is Likely Pathogenic because the reviewed evidence totals 8 points, below the Pathogenic threshold of ≥10. [19, 22, 25]</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" spans="1:18">
+      <c r="C17" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="82.8">
       <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17:7670656:CT&gt;C</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NM_000546.6:c.1052del (p.Lys351ArgfsTer19). MANE Select ENST00000269305.9. [6, 23, 24]</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">frameshift_variant</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Likely pathogenic; criteria provided, single submitter</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOT_FOUND (Does not mean AF=0). Exome and genome AF missing; re-query and r3 final review also report NOT_FOUND.</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">frameshift_variant; HIGH</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not applicable</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not applicable</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PVS1_Moderate. [22, 25]</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Moderate (+2 points). [22, 25]</t>
-        </is>
-      </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>The MANE frameshift p.Lys351ArgfsTer19 introduces a new stop at approximately residue 369. This stop falls within the Gly356–Asp393 branch of the TP53 PVS1 flowchart, with predicted NMD escape. [23–25]</t>
-        </is>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>The position of the new stop supports PVS1_Moderate rather than PVS1 at Very Strong strength. NOT_FOUND does not justify PM2. The resulting 2 points supports VUS under TP53 v2.4. [5, 22, 25]</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr">
-        <is>
-          <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; PVS1 flowchart [25]. ClinVar [20]: external comparison only.</t>
-        </is>
-      </c>
-      <c r="P18" s="4" t="inlineStr">
-        <is>
-          <t>Population frequencies are unavailable; NOT_FOUND does not establish absence. NMD escape is predicted. Functional, segregation and case-level evidence were not independently scored. [22–25]</t>
-        </is>
-      </c>
-      <c r="Q18" s="4" t="inlineStr">
-        <is>
-          <t>VUS — Variant of Uncertain Significance. PVS1_Moderate: 2 points under ClinGen TP53 v2.4. [22, 25]</t>
-        </is>
-      </c>
-      <c r="R18" s="4" t="inlineStr">
-        <is>
-          <t>ClinVar reports Likely Pathogenic. The project assessment remains VUS because PVS1_Moderate alone provides 2 points, insufficient for Likely Pathogenic. [20, 22, 25]</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:18">
+      <c r="C18" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="82.8">
       <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17:7675107:T&gt;C</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MANE Select: NM_000546.6
-ENST00000269305.9:c.505A&gt;G
-ENSP00000269305.4:p.Met169Val</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">missense_variant</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Uncertain significance; criteria provided, multiple submitters, no conflicts</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FOUND. Project gnomAD exome AF = 1.368095733867073e-6; genome AF unavailable. PM2_Supporting not assigned because ancestry-level counts/frequencies and quality information were not supplied. Missing AF is not zero. [7, 22, 23]</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">missense_variant; MODERATE</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tolerated</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NA (not available in project output)</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BS3_Supporting; BP4_Moderate. [22, 26, 27]</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BS3_Supporting: Supporting (−1 point). BP4_Moderate: Moderate (−2 points). Total = −3. [22]</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>ClinGen Table S3 reports M169V as partially functional in Kato and noLOF in Funk, Giacomelli and Kotler (BS3_Supporting). Table S2 reports aGVGD C0, BayesDel −0.0177298 and SpliceAI 0 (BP4_Moderate). [26, 27]</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>The functional results support BS3_Supporting (−1). BayesDel, aGVGD and SpliceAI meet BP4_Moderate (−2). The total of −3 supports Likely Benign under TP53 v2.4. SIFT was not counted separately; PM2 was not assigned from aggregate AF alone. [22, 26, 27]</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t>ACMG/AMP [5]; VEP [6]; gnomAD [7]; ClinGen TP53 v2.4 [22]; project annotation tables [23, 24]; functional Table S3 [26]; bioinformatic Table S2 [27]. ClinVar [21]: external comparison only.</t>
-        </is>
-      </c>
-      <c r="P19" s="4" t="inlineStr">
-        <is>
-          <t>ClinGen supplemental codes are preliminary and were checked against TP53 rule conditions. SpliceAI is predictive, not an RNA assay. No case-level evidence was scored. Additional evidence could change the assessment. [22, 26, 27]</t>
-        </is>
-      </c>
-      <c r="Q19" s="4" t="inlineStr">
-        <is>
-          <t>Likely Benign. BS3_Supporting (−1) + BP4_Moderate (−2) = −3 points under ClinGen TP53 v2.4. [22, 26, 27]</t>
-        </is>
-      </c>
-      <c r="R19" s="4" t="inlineStr">
-        <is>
-          <t>ClinVar project snapshot reports VUS. The project assessment is Likely Benign based on reviewed ClinGen functional and computational evidence. ClinVar was used only for comparison. [21, 22, 26, 27]</t>
-        </is>
+      <c r="C19" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -2940,7 +2997,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FFE049C-5577-4E8D-8D38-FF8A87E1BF85}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="B1:B32"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="64.69921875" customWidth="1"/>
@@ -3043,66 +3100,68 @@
       </c>
     </row>
     <row r="20" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[19] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 372539. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/372539/</t>
-        </is>
+      <c r="B20" s="16" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[20] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 1066207. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/1066207/</t>
-        </is>
+      <c r="B21" s="16" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="22" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[21] National Center for Biotechnology Information (NCBI). (n.d.). ClinVar: TP53 Variation ID 844926. Available at: https://www.ncbi.nlm.nih.gov/clinvar/variation/844926/</t>
-        </is>
+      <c r="B22" s="16" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="23" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[22] ClinGen TP53 Variant Curation Expert Panel. (n.d.). ClinGen TP53 Expert Panel specifications to the ACMG/AMP variant interpretation guidelines for TP53 (Version 2.4; GN009). Clinical Genome Resource. Retrieved October 24, 2026, from https://cspec.genome.network/cspec/ui/svi/svi/GN009</t>
-        </is>
+      <c r="B23" s="16" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="24" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[23] Graduation project team. (n.d.). Variant Prioritization + Scoring Final A [Unpublished project dataset and methodology]. Supplied ZIP archive. Sources: input/final_annotation_with_VEP_SIFT_PolyPhen.tsv; results/11_merged_VEP_ClinVar_gnomAD_CORRECTED.tsv; results/14_gnomad_r3_final_review.tsv; results/prioritized_variants_CORRECTED.tsv; docs/variant_prioritization_methods.md. Scores represent educational prioritization, not independent ACMG/AMP classifications.</t>
-        </is>
+      <c r="B24" s="16" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="25" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[24] Graduation project team. (n.d.). Graduation_Project_Final [Unpublished project annotation dataset]. Supplied ZIP archive. Sources: results/tables/clinvar_annotations.tsv; results/tables/final_annotation_with_VEP.tsv. ClinVar assertions are the project snapshots, not a live database reassessment.</t>
-        </is>
+      <c r="B25" s="16" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B26" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[25] ClinGen TP53 Variant Curation Expert Panel. (n.d.). PVS1 flowchart for TP53 null variants in relation to NM_000546.6 [Flowchart, Version 2.4 supporting file]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/a59085f9-6c52-4c36-9c42-159f3f2c3694/data</t>
-        </is>
+      <c r="B26" s="16" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="27" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[26] ClinGen TP53 Variant Curation Expert Panel. (n.d.). Supplementary Table S3: Functional results for selected assays and corresponding preliminary PS3 and BS3 codes for every possible p53 missense variant using the TP53 specifications v2 [Data set]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/f7b4de92-567a-497d-a8db-0f673c8bb36c/data</t>
-        </is>
+      <c r="B27" s="16" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="28" spans="2:2" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[27] ClinGen TP53 Variant Curation Expert Panel. (n.d.). Supplementary Table S2: Bioinformatic predictions and corresponding PP3 and BP4 codes for every possible p53 missense variant using the TP53 specifications v2 [Data set]. Clinical Genome Resource. https://cspec.genome.network/cspec/File/id/f24d9c2f-5cb4-4c1a-bdf6-7d73331fc77b/data</t>
-        </is>
+      <c r="B28" s="16" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" ht="27.6">
+      <c r="B29" s="12" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="12" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="12" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" ht="27.6">
+      <c r="B32" s="12" t="s">
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -3123,10 +3182,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="19"/>
     </row>
     <row r="3" spans="1:2" ht="42" customHeight="1">
       <c r="A3" s="5" t="s">

</xml_diff>